<commit_message>
May 30 - 13:00pm
</commit_message>
<xml_diff>
--- a/3.2 - project_emulators_detailed_final.xlsx
+++ b/3.2 - project_emulators_detailed_final.xlsx
@@ -10,16 +10,16 @@
     <sheet name="project_emulators_detailed" sheetId="1" r:id="rId1"/>
     <sheet name="project_emulators_detailed (2)" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="125725"/>
   <pivotCaches>
-    <pivotCache cacheId="17" r:id="rId3"/>
-    <pivotCache cacheId="19" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1516" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1530" uniqueCount="89">
   <si>
     <t>project</t>
   </si>
@@ -263,6 +263,30 @@
   <si>
     <t>Count of project</t>
   </si>
+  <si>
+    <t>Use low-overhead GPU emulation, improves compatibility and speed</t>
+  </si>
+  <si>
+    <t>Run emulator headless (no GUI), saves memory and CPU</t>
+  </si>
+  <si>
+    <t>Skip boot animation, speeds up boot time</t>
+  </si>
+  <si>
+    <t>Disable audio support, reduces CPU usage</t>
+  </si>
+  <si>
+    <t>Disable camera emulation, avoids failures and saves resources</t>
+  </si>
+  <si>
+    <t>Do not save snapshot on exit, reduces I/O load and speeds shutdown</t>
+  </si>
+  <si>
+    <t>emulator option</t>
+  </si>
+  <si>
+    <t>description</t>
+  </si>
 </sst>
 </file>
 
@@ -405,7 +429,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="34">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -585,6 +609,12 @@
         <bgColor indexed="65"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -746,13 +776,21 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -798,7 +836,50 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="6">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
 </styleSheet>
 </file>
@@ -5642,7 +5723,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="17" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="3" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="3" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="F2:G42" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" showAll="0"/>
@@ -5837,7 +5918,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="19" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="3" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="3" minRefreshableVersion="3" showCalcMbrs="0" useAutoFormatting="1" itemPrintTitles="1" createdVersion="3" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="F2:G42" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="3">
     <pivotField dataField="1" showAll="0"/>
@@ -6027,6 +6108,44 @@
   <dataFields count="1">
     <dataField name="Count of project" fld="0" subtotal="count" baseField="0" baseItem="0"/>
   </dataFields>
+  <formats count="4">
+    <format dxfId="5">
+      <pivotArea dataOnly="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1">
+            <x v="14"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="4">
+      <pivotArea dataOnly="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1">
+            <x v="15"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="3">
+      <pivotArea dataOnly="0" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1">
+            <x v="28"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+    <format dxfId="1">
+      <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
+        <references count="1">
+          <reference field="1" count="1">
+            <x v="26"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </format>
+  </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
 </pivotTableDefinition>
 </file>
@@ -11755,14 +11874,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G244"/>
+  <dimension ref="A1:K244"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="6" max="6" width="29.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -11773,7 +11893,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -11789,8 +11909,14 @@
       <c r="G2" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="J2" t="s">
+        <v>87</v>
+      </c>
+      <c r="K2" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -11806,8 +11932,14 @@
       <c r="G3" s="3">
         <v>36</v>
       </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="J3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="K3" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -11823,8 +11955,14 @@
       <c r="G4" s="3">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="J4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="K4" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -11840,8 +11978,14 @@
       <c r="G5" s="3">
         <v>34</v>
       </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="J5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="K5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11">
       <c r="A6" t="s">
         <v>3</v>
       </c>
@@ -11851,14 +11995,20 @@
       <c r="C6">
         <v>41</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G6" s="3">
+      <c r="G6" s="5">
         <v>33</v>
       </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="J6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="K6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11">
       <c r="A7" t="s">
         <v>3</v>
       </c>
@@ -11874,8 +12024,14 @@
       <c r="G7" s="3">
         <v>32</v>
       </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="J7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K7" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11">
       <c r="A8" t="s">
         <v>3</v>
       </c>
@@ -11885,14 +12041,20 @@
       <c r="C8">
         <v>41</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="6" t="s">
         <v>9</v>
       </c>
       <c r="G8" s="3">
         <v>29</v>
       </c>
-    </row>
-    <row r="9" spans="1:7">
+      <c r="J8" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="K8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -11909,7 +12071,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:11">
       <c r="A10" t="s">
         <v>12</v>
       </c>
@@ -11919,14 +12081,14 @@
       <c r="C10">
         <v>2</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="G10" s="5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11">
       <c r="A11" t="s">
         <v>12</v>
       </c>
@@ -11943,7 +12105,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:11">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -11953,14 +12115,14 @@
       <c r="C12">
         <v>2</v>
       </c>
-      <c r="F12" s="2" t="s">
+      <c r="F12" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G12" s="3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="G12" s="7">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -11977,7 +12139,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:11">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -11994,7 +12156,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7">
+    <row r="15" spans="1:11">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -12011,7 +12173,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:7">
+    <row r="16" spans="1:11">
       <c r="A16" t="s">
         <v>13</v>
       </c>
@@ -14692,5 +14854,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>